<commit_message>
+Premiere Ultra300 / BGA-484 : synthèse OK, placement OK, routage OK, 7ADC et 7DAC, structure filtre gain spectre haut et bas identique, +Toutes les IOs en 3.3V sauf pin d'horloge principale 1.8V +De nouveau des process synchrone dans les filtres FIR +Reset actif bas (vérifier le fonctionement Fast_to_Slow_CDC)
Ressource	Utilisé / total	%
4-LUT	28466 / 273408	11%
DFF	38273 / 273408	14%
XLUT	0 / 17088	0%
Carry 1-bit	14994 / 68352	22%
Register File block	28 / 1424	2%
CDC	0 / 1424	0%
Clock Buffer	0	-
Clock Switch	0 / 2848	0%
DSP	448 / 896	50%
Memory block	39 / 448	9%
WFG	2 / 70	3%
PLL	0 / 7	0%
GCK	42 / 80	53%
</commit_message>
<xml_diff>
--- a/script_NX/constraint/ULTRA300_BGA484_Pin_Configuration.xlsx
+++ b/script_NX/constraint/ULTRA300_BGA484_Pin_Configuration.xlsx
@@ -902,11 +902,6 @@
       <c r="K13" s="3" t="n"/>
       <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>i_config_clk</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
@@ -2061,11 +2056,6 @@
       <c r="K55" s="3" t="n"/>
       <c r="L55" s="3" t="n"/>
       <c r="M55" s="3" t="n"/>
-      <c r="N55" t="inlineStr">
-        <is>
-          <t>o_spectrum_bit</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
@@ -2092,11 +2082,6 @@
       <c r="K56" s="3" t="n"/>
       <c r="L56" s="3" t="n"/>
       <c r="M56" s="3" t="n"/>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>o_spectrum_wr_en</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -2123,11 +2108,6 @@
       <c r="K57" s="3" t="n"/>
       <c r="L57" s="3" t="n"/>
       <c r="M57" s="3" t="n"/>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>o_spectrum_clk</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -2154,11 +2134,6 @@
       <c r="K58" s="3" t="n"/>
       <c r="L58" s="3" t="n"/>
       <c r="M58" s="3" t="n"/>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>o_spectrum_sof</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
@@ -2211,11 +2186,6 @@
       <c r="K60" s="3" t="n"/>
       <c r="L60" s="3" t="n"/>
       <c r="M60" s="3" t="n"/>
-      <c r="N60" t="inlineStr">
-        <is>
-          <t>o_spectrum_sd_bit</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
@@ -2242,11 +2212,6 @@
       <c r="K61" s="3" t="n"/>
       <c r="L61" s="3" t="n"/>
       <c r="M61" s="3" t="n"/>
-      <c r="N61" t="inlineStr">
-        <is>
-          <t>o_spectrum_sd_wr_en</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
@@ -2273,11 +2238,6 @@
       <c r="K62" s="3" t="n"/>
       <c r="L62" s="3" t="n"/>
       <c r="M62" s="3" t="n"/>
-      <c r="N62" t="inlineStr">
-        <is>
-          <t>o_spectrum_sd_clk</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
@@ -2591,11 +2551,6 @@
       <c r="K73" s="3" t="n"/>
       <c r="L73" s="3" t="n"/>
       <c r="M73" s="3" t="n"/>
-      <c r="N73" t="inlineStr">
-        <is>
-          <t>i_reset</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -2830,11 +2785,6 @@
       <c r="K82" s="3" t="n"/>
       <c r="L82" s="3" t="n"/>
       <c r="M82" s="3" t="n"/>
-      <c r="N82" t="inlineStr">
-        <is>
-          <t>o_spectrum_sd_sof</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
@@ -3546,11 +3496,6 @@
       <c r="K108" s="3" t="n"/>
       <c r="L108" s="3" t="n"/>
       <c r="M108" s="3" t="n"/>
-      <c r="N108" t="inlineStr">
-        <is>
-          <t>i_config_bit</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
@@ -3577,11 +3522,6 @@
       <c r="K109" s="3" t="n"/>
       <c r="L109" s="3" t="n"/>
       <c r="M109" s="3" t="n"/>
-      <c r="N109" t="inlineStr">
-        <is>
-          <t>i_config_wr_en</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
@@ -3608,11 +3548,6 @@
       <c r="K110" s="3" t="n"/>
       <c r="L110" s="3" t="n"/>
       <c r="M110" s="3" t="n"/>
-      <c r="N110" t="inlineStr">
-        <is>
-          <t>i_config_sof</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
@@ -7257,6 +7192,11 @@
       <c r="K242" s="3" t="n"/>
       <c r="L242" s="3" t="n"/>
       <c r="M242" s="3" t="n"/>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>o_spectrum_sd_bit</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="3" t="inlineStr">
@@ -7283,6 +7223,11 @@
       <c r="K243" s="3" t="n"/>
       <c r="L243" s="3" t="n"/>
       <c r="M243" s="3" t="n"/>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>o_spectrum_sd_wr_en</t>
+        </is>
+      </c>
     </row>
     <row r="244" ht="30" customHeight="1">
       <c r="A244" s="3" t="inlineStr">
@@ -7887,6 +7832,11 @@
       <c r="K264" s="3" t="n"/>
       <c r="L264" s="3" t="n"/>
       <c r="M264" s="3" t="n"/>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>o_spectrum_sd_clk</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="3" t="inlineStr">
@@ -7913,6 +7863,11 @@
       <c r="K265" s="3" t="n"/>
       <c r="L265" s="3" t="n"/>
       <c r="M265" s="3" t="n"/>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>o_spectrum_sd_sof</t>
+        </is>
+      </c>
     </row>
     <row r="266" ht="30" customHeight="1">
       <c r="A266" s="3" t="inlineStr">
@@ -9128,6 +9083,11 @@
       <c r="K306" s="3" t="n"/>
       <c r="L306" s="3" t="n"/>
       <c r="M306" s="3" t="n"/>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>i_config_clk</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="3" t="inlineStr">
@@ -9154,6 +9114,11 @@
       <c r="K307" s="3" t="n"/>
       <c r="L307" s="3" t="n"/>
       <c r="M307" s="3" t="n"/>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>i_config_bit</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="3" t="inlineStr">
@@ -9180,6 +9145,11 @@
       <c r="K308" s="3" t="n"/>
       <c r="L308" s="3" t="n"/>
       <c r="M308" s="3" t="n"/>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>i_config_wr_en</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="3" t="inlineStr">
@@ -9206,6 +9176,11 @@
       <c r="K309" s="3" t="n"/>
       <c r="L309" s="3" t="n"/>
       <c r="M309" s="3" t="n"/>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>i_config_sof</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="3" t="inlineStr">
@@ -12832,6 +12807,11 @@
       <c r="K438" s="3" t="n"/>
       <c r="L438" s="3" t="n"/>
       <c r="M438" s="3" t="n"/>
+      <c r="N438" t="inlineStr">
+        <is>
+          <t>o_spectrum_bit</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="3" t="inlineStr">
@@ -12858,6 +12838,11 @@
       <c r="K439" s="3" t="n"/>
       <c r="L439" s="3" t="n"/>
       <c r="M439" s="3" t="n"/>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t>o_spectrum_wr_en</t>
+        </is>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="3" t="inlineStr">
@@ -12884,6 +12869,11 @@
       <c r="K440" s="3" t="n"/>
       <c r="L440" s="3" t="n"/>
       <c r="M440" s="3" t="n"/>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t>o_spectrum_clk</t>
+        </is>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="3" t="inlineStr">
@@ -12910,6 +12900,11 @@
       <c r="K441" s="3" t="n"/>
       <c r="L441" s="3" t="n"/>
       <c r="M441" s="3" t="n"/>
+      <c r="N441" t="inlineStr">
+        <is>
+          <t>o_spectrum_sof</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="3" t="inlineStr">

</xml_diff>